<commit_message>
proje kontrol listesi dolduruldu.
</commit_message>
<xml_diff>
--- a/docs/Proje__Kontrol_Listesi_482.xlsx
+++ b/docs/Proje__Kontrol_Listesi_482.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 1-2)</t>
+          <t>Delta_Design_Implementation_Report (s. 1-2)</t>
         </is>
       </c>
       <c r="D4" s="22" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md (s. 3-4)</t>
+          <t>SDD_v3 (s. 3-4)</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md, Test_Report_2026-04-16.md (s. 1-2, 1)</t>
+          <t>SDD_v3, Test_Report_2026-04-16 (s. 1-2, 1)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 1-2)</t>
+          <t>QUALITY_FACTORS (s. 1-2)</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 1-3)</t>
+          <t>Delta_Design_Implementation_Report (s. 1-3)</t>
         </is>
       </c>
       <c r="D8" s="22" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md (s. 2-3)</t>
+          <t>SDD_v3 (s. 2-3)</t>
         </is>
       </c>
       <c r="D9" s="22" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 2-3)</t>
+          <t>QUALITY_FACTORS (s. 2-3)</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 4-5)</t>
+          <t>Delta_Design_Implementation_Report (s. 4-5)</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md, Test_Report_2026-04-16.md (s. 1, 3)</t>
+          <t>SDD_v3, Test_Report_2026-04-16 (s. 1, 3)</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 2)</t>
+          <t>Delta_Design_Implementation_Report (s. 2)</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md (s. 3-4)</t>
+          <t>SDD_v3 (s. 3-4)</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Test_Report_2026-04-16.md (s. 3)</t>
+          <t>Test_Report_2026-04-16 (s. 3)</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md (s. 3-4)</t>
+          <t>SDD_v3 (s. 3-4)</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>SDD_v3.md (s. 2-3)</t>
+          <t>SDD_v3 (s. 2-3)</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 2-3)</t>
+          <t>QUALITY_FACTORS (s. 2-3)</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 4)</t>
+          <t>QUALITY_FACTORS (s. 4)</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 3-4)</t>
+          <t>Delta_Design_Implementation_Report (s. 3-4)</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 3)</t>
+          <t>QUALITY_FACTORS (s. 3)</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 3)</t>
+          <t>QUALITY_FACTORS (s. 3)</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 3)</t>
+          <t>QUALITY_FACTORS (s. 3)</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 5)</t>
+          <t>QUALITY_FACTORS (s. 5)</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 7)</t>
+          <t>QUALITY_FACTORS (s. 7)</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 1-2)</t>
+          <t>QUALITY_FACTORS (s. 1-2)</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 2)</t>
+          <t>Delta_Design_Implementation_Report (s. 2)</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 2), SDD_v3.md (s. 1)</t>
+          <t>Delta_Design_Implementation_Report (s. 2), SDD_v3 (s. 1)</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>Test_Report_2026-04-16.md (s. 2-3), QUALITY_FACTORS.md</t>
+          <t>Test_Report_2026-04-16 (s. 2-3), QUALITY_FACTORS</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>Test_Report_2026-04-16.md (s. 4-7)</t>
+          <t>Test_Report_2026-04-16 (s. 4-7)</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 1-2)</t>
+          <t>Delta_Design_Implementation_Report (s. 1-2)</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 3)</t>
+          <t>Delta_Design_Implementation_Report (s. 3)</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 1-2), Test_Report_2026-04-16.md (s. 6)</t>
+          <t>QUALITY_FACTORS (s. 1-2), Test_Report_2026-04-16 (s. 6)</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 3-4)</t>
+          <t>Delta_Design_Implementation_Report (s. 3-4)</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 2), SDD_v3.md (s. 1)</t>
+          <t>Delta_Design_Implementation_Report (s. 2), SDD_v3 (s. 1)</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C36" s="23" t="inlineStr">
         <is>
-          <t>Test_Report_2026-04-16.md (s. 2), QUALITY_FACTORS.md (s. 2)</t>
+          <t>Test_Report_2026-04-16 (s. 2), QUALITY_FACTORS (s. 2)</t>
         </is>
       </c>
       <c r="D36" s="23" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 1)</t>
+          <t>Delta_Design_Implementation_Report (s. 1)</t>
         </is>
       </c>
       <c r="D37" s="23" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C38" s="23" t="inlineStr">
         <is>
-          <t>Delta_Design_Implementation_Report.md (s. 2)</t>
+          <t>Delta_Design_Implementation_Report (s. 2)</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="C39" s="23" t="inlineStr">
         <is>
-          <t>QUALITY_FACTORS.md (s. 3), SDD_v3.md (s. 2)</t>
+          <t>QUALITY_FACTORS (s. 3), SDD_v3 (s. 2)</t>
         </is>
       </c>
       <c r="D39" s="23" t="inlineStr">

</xml_diff>